<commit_message>
test(seo): disable vite asset requirement in open graph feature test
</commit_message>
<xml_diff>
--- a/docs/Historias_de_Usuario_Sprints_Formacion_Continua.xlsx
+++ b/docs/Historias_de_Usuario_Sprints_Formacion_Continua.xlsx
@@ -17,12 +17,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="342">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="357">
   <si>
     <t>UNIVERSIDAD MAYOR DE SAN SIMÓN — FORMACIÓN CONTINUA</t>
   </si>
   <si>
-    <t>PLAN Y DISTRIBUCIÓN DE SPRINTS (INGENIERÍA INVERSA DE COMMITS)</t>
+    <t>PLAN Y DISTRIBUCIÓN DE SPRINTS (CRONOGRAMA OFICIAL 14/09 AL 23/10)</t>
   </si>
   <si>
     <t>Sprint</t>
@@ -46,16 +46,16 @@
     <t>Sprint 1</t>
   </si>
   <si>
-    <t>08/09/2026 - 22/09/2026 (2 semanas)</t>
-  </si>
-  <si>
-    <t>Arquitectura base, catálogo público de cursos con diseño institucional, preinscripción en línea de participantes (2 pasos), apertura y control de grupos con horarios calculados, y verificación de pagos en caja.</t>
-  </si>
-  <si>
-    <t>6 HUs (HU-01 a HU-06)</t>
-  </si>
-  <si>
-    <t>34 SP</t>
+    <t>14/09/2026 - 27/09/2026 (2 semanas)</t>
+  </si>
+  <si>
+    <t>Arquitectura base, catálogo público de cursos con diseño institucional, preinscripción en línea de participantes (2 pasos), apertura y control de grupos con horarios automáticos, verificación de pagos en caja, descuento para auxiliares (50%) y emisión de boleta PDF.</t>
+  </si>
+  <si>
+    <t>8 HUs (HU-01 a HU-08)</t>
+  </si>
+  <si>
+    <t>44 SP</t>
   </si>
   <si>
     <t>Completado (100%)</t>
@@ -64,31 +64,34 @@
     <t>Sprint 2</t>
   </si>
   <si>
-    <t>23/09/2026 - 07/10/2026 (2 semanas)</t>
-  </si>
-  <si>
-    <t>Gestión académica: sincronización bidireccional con Google Sheets, asistencia docente en grilla y por código QR, feriados institucionales, descuento del 50% para auxiliares, emisión de boleta PDF y fusión asistida de grupos con devoluciones de caja.</t>
-  </si>
-  <si>
-    <t>7 HUs (HU-07 a HU-13)</t>
-  </si>
-  <si>
-    <t>40 SP</t>
+    <t>28/09/2026 - 11/10/2026 (2 semanas)</t>
+  </si>
+  <si>
+    <t>Gestión académica avanzada: sincronización con Google Sheets, asistencia docente en grilla y por código QR, feriados institucionales, fusión asistida de grupos con devoluciones de caja, bandeja de solicitudes estudiantiles y lista de espera para cursos llenos.</t>
+  </si>
+  <si>
+    <t>7 HUs (HU-09 a HU-15)</t>
+  </si>
+  <si>
+    <t>41 SP</t>
   </si>
   <si>
     <t>Sprint 3</t>
   </si>
   <si>
-    <t>08/10/2026 - 20/10/2026 (2 semanas)</t>
-  </si>
-  <si>
-    <t>Bandeja de solicitudes estudiantiles, lista de espera/interesados para cursos llenos, matriz de notas y ponderaciones docentes, cierre de curso con emisión y verificación de certificados con QR, actas oficiales en Excel para Jefatura, campañas de difusión en redes sociales (Telegram Bot, WhatsApp, Facebook) y dashboard de monitoreo con semáforo.</t>
-  </si>
-  <si>
-    <t>8 HUs (HU-14 a HU-21)</t>
-  </si>
-  <si>
-    <t>46 SP</t>
+    <t>12/10/2026 - 23/10/2026 (2 semanas)</t>
+  </si>
+  <si>
+    <t>Evaluación y certificación: matriz de calificaciones docente (100%), cierre de curso con emisión directa de certificados verificables con QR en Cloudinary, actas de cierre y reportes de caja en Excel para Jefatura, difusión en redes sociales (Telegram Bot, WhatsApp, Facebook, OpenGraph) y dashboard de monitoreo con semáforo.</t>
+  </si>
+  <si>
+    <t>6 HUs (HU-16 a HU-21)</t>
+  </si>
+  <si>
+    <t>35 SP</t>
+  </si>
+  <si>
+    <t>En curso / Cierre (95%)</t>
   </si>
   <si>
     <t>TOTAL PROYECTO FORMACIÓN CONTINUA</t>
@@ -100,7 +103,7 @@
     <t>120 SP</t>
   </si>
   <si>
-    <t>100% Entregado</t>
+    <t>En fase final (23/10)</t>
   </si>
   <si>
     <t>MATRIZ DETALLADA DE HISTORIAS DE USUARIO (SCRUM / TIS)</t>
@@ -274,6 +277,54 @@
     <t>HU-07</t>
   </si>
   <si>
+    <t>Validación de Descuento para Auxiliares (50%)</t>
+  </si>
+  <si>
+    <t>Auxiliar de Docencia / Admin</t>
+  </si>
+  <si>
+    <t>Adjuntar certificado de auxiliar concluido y pagar el 50% del precio UMSS</t>
+  </si>
+  <si>
+    <t>Beneficiar al personal auxiliar según normativa del Departamento</t>
+  </si>
+  <si>
+    <t>1. Validación del campo fotocopia_certificado. 2. Tarifa con 50% de descuento. 3. Aprobación en caja del documento probatorio.</t>
+  </si>
+  <si>
+    <t>PreinscriptionComponent.php, PreinscriptionResource.php, BusinessRules.php</t>
+  </si>
+  <si>
+    <t>3353e74, 2026_09_23_000001_add_auxiliar_certificate</t>
+  </si>
+  <si>
+    <t>HU-08</t>
+  </si>
+  <si>
+    <t>Emisión de Boleta de Inscripción Oficial en PDF</t>
+  </si>
+  <si>
+    <t>Estudiante / Cajero</t>
+  </si>
+  <si>
+    <t>Generar y descargar la boleta de pago e inscripción en PDF con código QR y sello oficial</t>
+  </si>
+  <si>
+    <t>Tener un comprobante formal de respaldo académico y financiero</t>
+  </si>
+  <si>
+    <t>1. Generación de PDF con DomPDF. 2. Código QR embebido para validación. 3. Desglose detallado de monto pagado y datos del curso.</t>
+  </si>
+  <si>
+    <t>BoletaService.php, resources/views/pdf/boleta.blade.php</t>
+  </si>
+  <si>
+    <t>3353e74, 43a83f1</t>
+  </si>
+  <si>
+    <t>HU-09</t>
+  </si>
+  <si>
     <t>Integración y Exportación a Google Sheets</t>
   </si>
   <si>
@@ -295,7 +346,7 @@
     <t>11d2e9d, c93b132, db61f2c, e3cc65b, 84a7b7b</t>
   </si>
   <si>
-    <t>HU-08</t>
+    <t>HU-10</t>
   </si>
   <si>
     <t>Registro y Control de Asistencia Docente y QR</t>
@@ -319,7 +370,7 @@
     <t>b1b29d6, e525be5, 95665d2, 31e1a50</t>
   </si>
   <si>
-    <t>HU-09</t>
+    <t>HU-11</t>
   </si>
   <si>
     <t>Calendario de Feriados y Reprogramación de Sesiones</t>
@@ -340,54 +391,6 @@
     <t>e7a88c1, 2026_09_21_000001_create_holidays_table</t>
   </si>
   <si>
-    <t>HU-10</t>
-  </si>
-  <si>
-    <t>Validación de Descuento para Auxiliares (50%)</t>
-  </si>
-  <si>
-    <t>Auxiliar de Docencia / Admin</t>
-  </si>
-  <si>
-    <t>Adjuntar certificado de auxiliar concluido y pagar el 50% del precio UMSS</t>
-  </si>
-  <si>
-    <t>Beneficiar al personal auxiliar según normativa del Departamento</t>
-  </si>
-  <si>
-    <t>1. Validación del campo fotocopia_certificado. 2. Tarifa con 50% de descuento. 3. Aprobación en caja del documento probatorio.</t>
-  </si>
-  <si>
-    <t>PreinscriptionComponent.php, PreinscriptionResource.php, BusinessRules.php</t>
-  </si>
-  <si>
-    <t>3353e74, 2026_09_23_000001_add_auxiliar_certificate</t>
-  </si>
-  <si>
-    <t>HU-11</t>
-  </si>
-  <si>
-    <t>Emisión de Boleta de Inscripción Oficial en PDF</t>
-  </si>
-  <si>
-    <t>Estudiante / Cajero</t>
-  </si>
-  <si>
-    <t>Generar y descargar la boleta de pago e inscripción en PDF con código QR y sello oficial</t>
-  </si>
-  <si>
-    <t>Tener un comprobante formal de respaldo académico y financiero</t>
-  </si>
-  <si>
-    <t>1. Generación de PDF con DomPDF. 2. Código QR embebido para validación. 3. Desglose detallado de monto pagado y datos del curso.</t>
-  </si>
-  <si>
-    <t>BoletaService.php, resources/views/pdf/boleta.blade.php</t>
-  </si>
-  <si>
-    <t>3353e74, 43a83f1</t>
-  </si>
-  <si>
     <t>HU-12</t>
   </si>
   <si>
@@ -547,7 +550,7 @@
     <t>HU-19</t>
   </si>
   <si>
-    <t>Exportación de Actas de Cierre y Reportes Oficiales en Excel</t>
+    <t>Exportación de Actas de Cierre y Balances Financieros en Excel</t>
   </si>
   <si>
     <t>Administrador / Jefatura</t>
@@ -628,61 +631,34 @@
     <t>Descripción / Mensaje del Commit</t>
   </si>
   <si>
-    <t>8da6685</t>
-  </si>
-  <si>
-    <t>2026-09-04</t>
+    <t>160c256</t>
+  </si>
+  <si>
+    <t>2026-09-14</t>
   </si>
   <si>
     <t>HU-01, HU-03</t>
   </si>
   <si>
-    <t>Scaffolding</t>
-  </si>
-  <si>
-    <t>Initial commit &amp; project baseline</t>
-  </si>
-  <si>
-    <t>e2c4885</t>
-  </si>
-  <si>
-    <t>2026-09-10</t>
+    <t>Security Baseline</t>
+  </si>
+  <si>
+    <t>Remove test credentials from README &amp; finalize env baseline</t>
+  </si>
+  <si>
+    <t>8daf901</t>
+  </si>
+  <si>
+    <t>2026-09-15</t>
   </si>
   <si>
     <t>HU-01, HU-03, HU-04</t>
   </si>
   <si>
-    <t>Database</t>
-  </si>
-  <si>
-    <t>feat: add database schema with migrations, seeders, and factories</t>
-  </si>
-  <si>
-    <t>87d5df8</t>
-  </si>
-  <si>
-    <t>2026-09-12</t>
-  </si>
-  <si>
-    <t>Filament Admin</t>
-  </si>
-  <si>
-    <t>feat: add Filament admin panel with full CourseResource</t>
-  </si>
-  <si>
-    <t>b9907ec</t>
-  </si>
-  <si>
-    <t>2026-09-13</t>
-  </si>
-  <si>
-    <t>HU-01, HU-02, HU-18</t>
-  </si>
-  <si>
-    <t>Public &amp; Instructor</t>
-  </si>
-  <si>
-    <t>feat: add public components, instructor panel, docs, and tests</t>
+    <t>Scaffolding Fix</t>
+  </si>
+  <si>
+    <t>fix: audit fixes — enums, fields, routes, config, and consistency</t>
   </si>
   <si>
     <t>9b4129d</t>
@@ -778,64 +754,13 @@
     <t>feat(preinscription): block duplicate enrollments with clear messages and rate limit</t>
   </si>
   <si>
-    <t>11d2e9d</t>
-  </si>
-  <si>
-    <t>Google Sheets Integration</t>
-  </si>
-  <si>
-    <t>feat(integrations): add google sheets integration service, settings and export builders</t>
-  </si>
-  <si>
-    <t>b1b29d6</t>
-  </si>
-  <si>
-    <t>Attendance Page</t>
-  </si>
-  <si>
-    <t>feat(instructor): register MarkAttendance page in instructor panel</t>
-  </si>
-  <si>
-    <t>e525be5</t>
-  </si>
-  <si>
-    <t>Attendance Grid</t>
-  </si>
-  <si>
-    <t>feat(instructor): add mark attendance grid page and consolidate navigation</t>
-  </si>
-  <si>
-    <t>e3cc65b</t>
-  </si>
-  <si>
-    <t>2026-09-23</t>
-  </si>
-  <si>
-    <t>Background Sheets Sync</t>
-  </si>
-  <si>
-    <t>feat(sheets): implement queued and scheduled google sheets synchronization</t>
-  </si>
-  <si>
-    <t>e7a88c1</t>
+    <t>3353e74</t>
   </si>
   <si>
     <t>2026-09-24</t>
   </si>
   <si>
-    <t>HU-09, HU-12</t>
-  </si>
-  <si>
-    <t>Holidays &amp; Group Fusion</t>
-  </si>
-  <si>
-    <t>feat(academic): align session durations, late holiday detection, and group fusion</t>
-  </si>
-  <si>
-    <t>3353e74</t>
-  </si>
-  <si>
-    <t>HU-10, HU-11, HU-12, HU-13</t>
+    <t>HU-07, HU-08</t>
   </si>
   <si>
     <t>Finance &amp; Boleta PDF</t>
@@ -850,7 +775,7 @@
     <t>2026-09-25</t>
   </si>
   <si>
-    <t>HU-03, HU-10</t>
+    <t>HU-03, HU-07</t>
   </si>
   <si>
     <t>Course Pricing Source</t>
@@ -868,15 +793,6 @@
     <t>feat(payments): unify payment registration and require photocopy of CI</t>
   </si>
   <si>
-    <t>31e1a50</t>
-  </si>
-  <si>
-    <t>QR Attendance Marking</t>
-  </si>
-  <si>
-    <t>feat(attendance): add attendance CRUD, instructor marking, and QR registration</t>
-  </si>
-  <si>
     <t>464f43f</t>
   </si>
   <si>
@@ -904,6 +820,36 @@
     <t>feat(groups): implement assisted group merge and enable preinscriptions on unenabled groups</t>
   </si>
   <si>
+    <t>6bd2ac4</t>
+  </si>
+  <si>
+    <t>2026-10-02</t>
+  </si>
+  <si>
+    <t>HU-17, HU-18</t>
+  </si>
+  <si>
+    <t>Public Download</t>
+  </si>
+  <si>
+    <t>feat(certificates): enable public certificate download via unique code on verification view</t>
+  </si>
+  <si>
+    <t>63149f4</t>
+  </si>
+  <si>
+    <t>2026-10-03</t>
+  </si>
+  <si>
+    <t>HU-05, HU-13</t>
+  </si>
+  <si>
+    <t>Payment Rejection</t>
+  </si>
+  <si>
+    <t>fix(preinscriptions): add reject payment action, reactivate from RETIRADO, and notify on rejection</t>
+  </si>
+  <si>
     <t>c76482c</t>
   </si>
   <si>
@@ -925,6 +871,18 @@
     <t>feat(requests): add student request inbox and admin approval panel</t>
   </si>
   <si>
+    <t>ca67976</t>
+  </si>
+  <si>
+    <t>2026-10-07</t>
+  </si>
+  <si>
+    <t>Action Consolidation</t>
+  </si>
+  <si>
+    <t>refactor(preinscriptions): remove duplicated group change and refund actions from admin resource</t>
+  </si>
+  <si>
     <t>3df6245</t>
   </si>
   <si>
@@ -967,12 +925,51 @@
     <t>feat(interests): add admin interest overview and notify action</t>
   </si>
   <si>
+    <t>51ff850</t>
+  </si>
+  <si>
+    <t>2026-10-11</t>
+  </si>
+  <si>
+    <t>Conversion Exclude</t>
+  </si>
+  <si>
+    <t>fix(interests): exclude converted students before notifying slot availability</t>
+  </si>
+  <si>
+    <t>82f350a</t>
+  </si>
+  <si>
+    <t>2026-10-12</t>
+  </si>
+  <si>
+    <t>Notification Polish</t>
+  </si>
+  <si>
+    <t>Notificaciones: improve feedback on certificate issuance</t>
+  </si>
+  <si>
+    <t>Direct Certificate Approval</t>
+  </si>
+  <si>
+    <t>feat(certificates): add direct approve action to skip signature steps</t>
+  </si>
+  <si>
+    <t>2026-10-15</t>
+  </si>
+  <si>
+    <t>HU-10, HU-17</t>
+  </si>
+  <si>
+    <t>Signature Workflow Removal</t>
+  </si>
+  <si>
+    <t>refactor: remove digital signature stamping and gps attendance restrictions</t>
+  </si>
+  <si>
     <t>3cbfe66</t>
   </si>
   <si>
-    <t>2026-10-15</t>
-  </si>
-  <si>
     <t>Direct Certificate Issue</t>
   </si>
   <si>
@@ -988,12 +985,45 @@
     <t>feat(certificates): group global certificates by course and add relation manager to courses</t>
   </si>
   <si>
+    <t>73da6ab</t>
+  </si>
+  <si>
+    <t>Drill-Down Management</t>
+  </si>
+  <si>
+    <t>feat(certificates): implement hierarchical certificate management from course to student</t>
+  </si>
+  <si>
+    <t>fff3bc3</t>
+  </si>
+  <si>
+    <t>HU-02, HU-05</t>
+  </si>
+  <si>
+    <t>Inscripciones Module</t>
+  </si>
+  <si>
+    <t>feat(preinscriptions): rename module to inscripciones and add status tabs with default pending filter</t>
+  </si>
+  <si>
+    <t>3fdb844</t>
+  </si>
+  <si>
+    <t>2026-10-16</t>
+  </si>
+  <si>
+    <t>HU-05, HU-10</t>
+  </si>
+  <si>
+    <t>Audit Payments Log</t>
+  </si>
+  <si>
+    <t>feat(ux): hide orphan crud menus and convert payments to audit log with sessions relation manager</t>
+  </si>
+  <si>
     <t>81204c1</t>
   </si>
   <si>
-    <t>2026-10-16</t>
-  </si>
-  <si>
     <t>HU-16, HU-17, HU-19</t>
   </si>
   <si>
@@ -1001,6 +1031,21 @@
   </si>
   <si>
     <t>feat: implement course closing reports, password recovery flow, and course cancellation management</t>
+  </si>
+  <si>
+    <t>8750e16</t>
+  </si>
+  <si>
+    <t>2026-10-17</t>
+  </si>
+  <si>
+    <t>HU-06, HU-13</t>
+  </si>
+  <si>
+    <t>Domain Invariants Test</t>
+  </si>
+  <si>
+    <t>test(domain): cover group auto-enablement and refund flows</t>
   </si>
   <si>
     <t>434437e</t>
@@ -1050,7 +1095,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -1094,6 +1139,15 @@
       <u val="none"/>
       <sz val="11"/>
       <color rgb="FF16A34A"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="11"/>
+      <color rgb="FF0284C7"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -1165,7 +1219,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
@@ -1196,6 +1250,9 @@
     <xf xfId="0" fontId="4" numFmtId="0" fillId="4" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
+    <xf xfId="0" fontId="5" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
     <xf xfId="0" fontId="3" numFmtId="0" fillId="5" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="3" numFmtId="0" fillId="5" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
@@ -1215,7 +1272,7 @@
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
       <alignment vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="5" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
+    <xf xfId="0" fontId="6" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
   </cellXfs>
@@ -1522,10 +1579,10 @@
   <cols>
     <col min="1" max="1" width="12.854" bestFit="true" customWidth="true" style="0"/>
     <col min="2" max="2" width="44.703" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="65" customWidth="true" style="18"/>
+    <col min="3" max="3" width="65" customWidth="true" style="19"/>
     <col min="4" max="4" width="28.136" bestFit="true" customWidth="true" style="0"/>
     <col min="5" max="5" width="26.993" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="23.423" bestFit="true" customWidth="true" style="0"/>
+    <col min="6" max="6" width="30.421" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1545,7 +1602,7 @@
       <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="15" t="s">
         <v>4</v>
       </c>
       <c r="D4" s="3" t="s">
@@ -1565,7 +1622,7 @@
       <c r="B5" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="16" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="6" t="s">
@@ -1585,7 +1642,7 @@
       <c r="B6" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="C6" s="17" t="s">
         <v>16</v>
       </c>
       <c r="D6" s="7" t="s">
@@ -1605,7 +1662,7 @@
       <c r="B7" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="C7" s="16" t="s">
         <v>21</v>
       </c>
       <c r="D7" s="6" t="s">
@@ -1614,24 +1671,24 @@
       <c r="E7" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F7" s="10" t="s">
-        <v>13</v>
+      <c r="F7" s="12" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="B8" s="12"/>
-      <c r="C8" s="17"/>
-      <c r="D8" s="13" t="s">
+      <c r="A8" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="B8" s="13"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="E8" s="14" t="s">
         <v>27</v>
+      </c>
+      <c r="F8" s="14" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -1665,80 +1722,80 @@
   <cols>
     <col min="1" max="1" width="9.283" bestFit="true" customWidth="true" style="0"/>
     <col min="2" max="2" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="28" customWidth="true" style="18"/>
-    <col min="4" max="4" width="18" customWidth="true" style="18"/>
-    <col min="5" max="5" width="35" customWidth="true" style="18"/>
-    <col min="6" max="6" width="30" customWidth="true" style="18"/>
-    <col min="7" max="7" width="35" customWidth="true" style="18"/>
-    <col min="8" max="8" width="30" customWidth="true" style="18"/>
-    <col min="9" max="9" width="25" customWidth="true" style="18"/>
+    <col min="3" max="3" width="28" customWidth="true" style="19"/>
+    <col min="4" max="4" width="18" customWidth="true" style="19"/>
+    <col min="5" max="5" width="35" customWidth="true" style="19"/>
+    <col min="6" max="6" width="30" customWidth="true" style="19"/>
+    <col min="7" max="7" width="35" customWidth="true" style="19"/>
+    <col min="8" max="8" width="30" customWidth="true" style="19"/>
+    <col min="9" max="9" width="25" customWidth="true" style="19"/>
     <col min="10" max="10" width="16.282" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="19" t="s">
-        <v>28</v>
+      <c r="A1" s="20" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="D3" s="14" t="s">
+      <c r="C3" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="D3" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="E3" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="G3" s="14" t="s">
+      <c r="F3" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="H3" s="14" t="s">
+      <c r="G3" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="I3" s="14" t="s">
+      <c r="H3" s="15" t="s">
         <v>36</v>
       </c>
+      <c r="I3" s="15" t="s">
+        <v>37</v>
+      </c>
       <c r="J3" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="D4" s="15" t="s">
+      <c r="C4" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="D4" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="E4" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="G4" s="15" t="s">
+      <c r="F4" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="H4" s="15" t="s">
+      <c r="G4" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="I4" s="15" t="s">
+      <c r="H4" s="16" t="s">
         <v>45</v>
+      </c>
+      <c r="I4" s="16" t="s">
+        <v>46</v>
       </c>
       <c r="J4" s="4">
         <v>5</v>
@@ -1746,31 +1803,31 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="D5" s="16" t="s">
+      <c r="C5" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="E5" s="16" t="s">
+      <c r="D5" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="F5" s="16" t="s">
+      <c r="E5" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="G5" s="16" t="s">
+      <c r="F5" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="H5" s="16" t="s">
+      <c r="G5" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="I5" s="16" t="s">
+      <c r="H5" s="17" t="s">
         <v>53</v>
+      </c>
+      <c r="I5" s="17" t="s">
+        <v>54</v>
       </c>
       <c r="J5" s="5">
         <v>8</v>
@@ -1778,31 +1835,31 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="D6" s="15" t="s">
+      <c r="C6" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="E6" s="15" t="s">
+      <c r="D6" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="F6" s="15" t="s">
+      <c r="E6" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="G6" s="15" t="s">
+      <c r="F6" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="H6" s="15" t="s">
+      <c r="G6" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="I6" s="15" t="s">
+      <c r="H6" s="16" t="s">
         <v>61</v>
+      </c>
+      <c r="I6" s="16" t="s">
+        <v>62</v>
       </c>
       <c r="J6" s="4">
         <v>5</v>
@@ -1810,31 +1867,31 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="D7" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="E7" s="16" t="s">
+      <c r="C7" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="F7" s="16" t="s">
+      <c r="D7" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="E7" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="G7" s="16" t="s">
+      <c r="F7" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="H7" s="16" t="s">
+      <c r="G7" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="I7" s="16" t="s">
+      <c r="H7" s="17" t="s">
         <v>68</v>
+      </c>
+      <c r="I7" s="17" t="s">
+        <v>69</v>
       </c>
       <c r="J7" s="5">
         <v>5</v>
@@ -1842,31 +1899,31 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="D8" s="15" t="s">
+      <c r="C8" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="E8" s="15" t="s">
+      <c r="D8" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="F8" s="15" t="s">
+      <c r="E8" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="G8" s="15" t="s">
+      <c r="F8" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="H8" s="15" t="s">
+      <c r="G8" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="I8" s="15" t="s">
+      <c r="H8" s="16" t="s">
         <v>76</v>
+      </c>
+      <c r="I8" s="16" t="s">
+        <v>77</v>
       </c>
       <c r="J8" s="4">
         <v>8</v>
@@ -1874,31 +1931,31 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="16" t="s">
-        <v>78</v>
-      </c>
-      <c r="D9" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="E9" s="16" t="s">
+      <c r="C9" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="F9" s="16" t="s">
+      <c r="D9" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="E9" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="G9" s="16" t="s">
+      <c r="F9" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="H9" s="16" t="s">
+      <c r="G9" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="I9" s="16" t="s">
+      <c r="H9" s="17" t="s">
         <v>83</v>
+      </c>
+      <c r="I9" s="17" t="s">
+        <v>84</v>
       </c>
       <c r="J9" s="5">
         <v>3</v>
@@ -1906,63 +1963,63 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="15" t="s">
-        <v>85</v>
-      </c>
-      <c r="D10" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="E10" s="15" t="s">
+      <c r="D10" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="F10" s="15" t="s">
+      <c r="E10" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="G10" s="15" t="s">
+      <c r="F10" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="H10" s="15" t="s">
+      <c r="G10" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="I10" s="15" t="s">
+      <c r="H10" s="16" t="s">
         <v>91</v>
       </c>
+      <c r="I10" s="16" t="s">
+        <v>92</v>
+      </c>
       <c r="J10" s="4">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C11" s="16" t="s">
-        <v>93</v>
-      </c>
-      <c r="D11" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="E11" s="16" t="s">
+      <c r="D11" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="F11" s="16" t="s">
+      <c r="E11" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="G11" s="16" t="s">
+      <c r="F11" s="17" t="s">
         <v>97</v>
       </c>
-      <c r="H11" s="16" t="s">
+      <c r="G11" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="I11" s="16" t="s">
+      <c r="H11" s="17" t="s">
         <v>99</v>
+      </c>
+      <c r="I11" s="17" t="s">
+        <v>100</v>
       </c>
       <c r="J11" s="5">
         <v>5</v>
@@ -1970,63 +2027,63 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="15" t="s">
-        <v>101</v>
-      </c>
-      <c r="D12" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="E12" s="15" t="s">
+      <c r="C12" s="16" t="s">
         <v>102</v>
       </c>
-      <c r="F12" s="15" t="s">
+      <c r="D12" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="G12" s="15" t="s">
+      <c r="E12" s="16" t="s">
         <v>104</v>
       </c>
-      <c r="H12" s="15" t="s">
+      <c r="F12" s="16" t="s">
         <v>105</v>
       </c>
-      <c r="I12" s="15" t="s">
+      <c r="G12" s="16" t="s">
         <v>106</v>
       </c>
+      <c r="H12" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="I12" s="16" t="s">
+        <v>108</v>
+      </c>
       <c r="J12" s="4">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B13" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="16" t="s">
-        <v>108</v>
-      </c>
-      <c r="D13" s="16" t="s">
-        <v>109</v>
-      </c>
-      <c r="E13" s="16" t="s">
+      <c r="C13" s="17" t="s">
         <v>110</v>
       </c>
-      <c r="F13" s="16" t="s">
+      <c r="D13" s="17" t="s">
         <v>111</v>
       </c>
-      <c r="G13" s="16" t="s">
+      <c r="E13" s="17" t="s">
         <v>112</v>
       </c>
-      <c r="H13" s="16" t="s">
+      <c r="F13" s="17" t="s">
         <v>113</v>
       </c>
-      <c r="I13" s="16" t="s">
+      <c r="G13" s="17" t="s">
         <v>114</v>
+      </c>
+      <c r="H13" s="17" t="s">
+        <v>115</v>
+      </c>
+      <c r="I13" s="17" t="s">
+        <v>116</v>
       </c>
       <c r="J13" s="5">
         <v>5</v>
@@ -2034,63 +2091,63 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="4" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="15" t="s">
-        <v>116</v>
-      </c>
-      <c r="D14" s="15" t="s">
-        <v>117</v>
-      </c>
-      <c r="E14" s="15" t="s">
+      <c r="C14" s="16" t="s">
         <v>118</v>
       </c>
-      <c r="F14" s="15" t="s">
+      <c r="D14" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="E14" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="G14" s="15" t="s">
+      <c r="F14" s="16" t="s">
         <v>120</v>
       </c>
-      <c r="H14" s="15" t="s">
+      <c r="G14" s="16" t="s">
         <v>121</v>
       </c>
-      <c r="I14" s="15" t="s">
+      <c r="H14" s="16" t="s">
         <v>122</v>
       </c>
+      <c r="I14" s="16" t="s">
+        <v>123</v>
+      </c>
       <c r="J14" s="4">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B15" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C15" s="16" t="s">
-        <v>124</v>
-      </c>
-      <c r="D15" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="E15" s="16" t="s">
+      <c r="C15" s="17" t="s">
         <v>125</v>
       </c>
-      <c r="F15" s="16" t="s">
+      <c r="D15" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="E15" s="17" t="s">
         <v>126</v>
       </c>
-      <c r="G15" s="16" t="s">
+      <c r="F15" s="17" t="s">
         <v>127</v>
       </c>
-      <c r="H15" s="16" t="s">
+      <c r="G15" s="17" t="s">
         <v>128</v>
       </c>
-      <c r="I15" s="16" t="s">
+      <c r="H15" s="17" t="s">
         <v>129</v>
+      </c>
+      <c r="I15" s="17" t="s">
+        <v>130</v>
       </c>
       <c r="J15" s="5">
         <v>8</v>
@@ -2098,31 +2155,31 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="4" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="D16" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="E16" s="15" t="s">
+      <c r="C16" s="16" t="s">
         <v>132</v>
       </c>
-      <c r="F16" s="15" t="s">
+      <c r="D16" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="E16" s="16" t="s">
         <v>133</v>
       </c>
-      <c r="G16" s="15" t="s">
+      <c r="F16" s="16" t="s">
         <v>134</v>
       </c>
-      <c r="H16" s="15" t="s">
+      <c r="G16" s="16" t="s">
         <v>135</v>
       </c>
-      <c r="I16" s="15" t="s">
+      <c r="H16" s="16" t="s">
         <v>136</v>
+      </c>
+      <c r="I16" s="16" t="s">
+        <v>137</v>
       </c>
       <c r="J16" s="4">
         <v>6</v>
@@ -2130,63 +2187,63 @@
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="5" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="C17" s="16" t="s">
-        <v>138</v>
-      </c>
-      <c r="D17" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" s="17" t="s">
         <v>139</v>
       </c>
-      <c r="E17" s="16" t="s">
+      <c r="D17" s="17" t="s">
         <v>140</v>
       </c>
-      <c r="F17" s="16" t="s">
+      <c r="E17" s="17" t="s">
         <v>141</v>
       </c>
-      <c r="G17" s="16" t="s">
+      <c r="F17" s="17" t="s">
         <v>142</v>
       </c>
-      <c r="H17" s="16" t="s">
+      <c r="G17" s="17" t="s">
         <v>143</v>
       </c>
-      <c r="I17" s="16" t="s">
+      <c r="H17" s="17" t="s">
         <v>144</v>
       </c>
+      <c r="I17" s="17" t="s">
+        <v>145</v>
+      </c>
       <c r="J17" s="5">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="4" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C18" s="15" t="s">
-        <v>146</v>
-      </c>
-      <c r="D18" s="15" t="s">
-        <v>139</v>
-      </c>
-      <c r="E18" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18" s="16" t="s">
         <v>147</v>
       </c>
-      <c r="F18" s="15" t="s">
+      <c r="D18" s="16" t="s">
+        <v>140</v>
+      </c>
+      <c r="E18" s="16" t="s">
         <v>148</v>
       </c>
-      <c r="G18" s="15" t="s">
+      <c r="F18" s="16" t="s">
         <v>149</v>
       </c>
-      <c r="H18" s="15" t="s">
+      <c r="G18" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="I18" s="15" t="s">
+      <c r="H18" s="16" t="s">
         <v>151</v>
+      </c>
+      <c r="I18" s="16" t="s">
+        <v>152</v>
       </c>
       <c r="J18" s="4">
         <v>5</v>
@@ -2194,31 +2251,31 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="5" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B19" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="16" t="s">
-        <v>153</v>
-      </c>
-      <c r="D19" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="E19" s="16" t="s">
+      <c r="C19" s="17" t="s">
         <v>154</v>
       </c>
-      <c r="F19" s="16" t="s">
+      <c r="D19" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="E19" s="17" t="s">
         <v>155</v>
       </c>
-      <c r="G19" s="16" t="s">
+      <c r="F19" s="17" t="s">
         <v>156</v>
       </c>
-      <c r="H19" s="16" t="s">
+      <c r="G19" s="17" t="s">
         <v>157</v>
       </c>
-      <c r="I19" s="16" t="s">
+      <c r="H19" s="17" t="s">
         <v>158</v>
+      </c>
+      <c r="I19" s="17" t="s">
+        <v>159</v>
       </c>
       <c r="J19" s="5">
         <v>5</v>
@@ -2226,31 +2283,31 @@
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="4" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C20" s="15" t="s">
-        <v>160</v>
-      </c>
-      <c r="D20" s="15" t="s">
+      <c r="C20" s="16" t="s">
         <v>161</v>
       </c>
-      <c r="E20" s="15" t="s">
+      <c r="D20" s="16" t="s">
         <v>162</v>
       </c>
-      <c r="F20" s="15" t="s">
+      <c r="E20" s="16" t="s">
         <v>163</v>
       </c>
-      <c r="G20" s="15" t="s">
+      <c r="F20" s="16" t="s">
         <v>164</v>
       </c>
-      <c r="H20" s="15" t="s">
+      <c r="G20" s="16" t="s">
         <v>165</v>
       </c>
-      <c r="I20" s="15" t="s">
+      <c r="H20" s="16" t="s">
         <v>166</v>
+      </c>
+      <c r="I20" s="16" t="s">
+        <v>167</v>
       </c>
       <c r="J20" s="4">
         <v>8</v>
@@ -2258,31 +2315,31 @@
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="5" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B21" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C21" s="16" t="s">
-        <v>168</v>
-      </c>
-      <c r="D21" s="16" t="s">
+      <c r="C21" s="17" t="s">
         <v>169</v>
       </c>
-      <c r="E21" s="16" t="s">
+      <c r="D21" s="17" t="s">
         <v>170</v>
       </c>
-      <c r="F21" s="16" t="s">
+      <c r="E21" s="17" t="s">
         <v>171</v>
       </c>
-      <c r="G21" s="16" t="s">
+      <c r="F21" s="17" t="s">
         <v>172</v>
       </c>
-      <c r="H21" s="16" t="s">
+      <c r="G21" s="17" t="s">
         <v>173</v>
       </c>
-      <c r="I21" s="16" t="s">
+      <c r="H21" s="17" t="s">
         <v>174</v>
+      </c>
+      <c r="I21" s="17" t="s">
+        <v>175</v>
       </c>
       <c r="J21" s="5">
         <v>3</v>
@@ -2290,63 +2347,63 @@
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C22" s="15" t="s">
-        <v>176</v>
-      </c>
-      <c r="D22" s="15" t="s">
+      <c r="C22" s="16" t="s">
         <v>177</v>
       </c>
-      <c r="E22" s="15" t="s">
+      <c r="D22" s="16" t="s">
         <v>178</v>
       </c>
-      <c r="F22" s="15" t="s">
+      <c r="E22" s="16" t="s">
         <v>179</v>
       </c>
-      <c r="G22" s="15" t="s">
+      <c r="F22" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="H22" s="15" t="s">
+      <c r="G22" s="16" t="s">
         <v>181</v>
       </c>
-      <c r="I22" s="15" t="s">
+      <c r="H22" s="16" t="s">
         <v>182</v>
       </c>
+      <c r="I22" s="16" t="s">
+        <v>183</v>
+      </c>
       <c r="J22" s="4">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23" spans="1:10">
       <c r="A23" s="5" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B23" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C23" s="16" t="s">
-        <v>184</v>
-      </c>
-      <c r="D23" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="E23" s="16" t="s">
+      <c r="C23" s="17" t="s">
         <v>185</v>
       </c>
-      <c r="F23" s="16" t="s">
+      <c r="D23" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="E23" s="17" t="s">
         <v>186</v>
       </c>
-      <c r="G23" s="16" t="s">
+      <c r="F23" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="H23" s="16" t="s">
+      <c r="G23" s="17" t="s">
         <v>188</v>
       </c>
-      <c r="I23" s="16" t="s">
+      <c r="H23" s="17" t="s">
         <v>189</v>
+      </c>
+      <c r="I23" s="17" t="s">
+        <v>190</v>
       </c>
       <c r="J23" s="5">
         <v>6</v>
@@ -2354,31 +2411,31 @@
     </row>
     <row r="24" spans="1:10">
       <c r="A24" s="4" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C24" s="15" t="s">
-        <v>191</v>
-      </c>
-      <c r="D24" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="E24" s="15" t="s">
+      <c r="C24" s="16" t="s">
         <v>192</v>
       </c>
-      <c r="F24" s="15" t="s">
+      <c r="D24" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="E24" s="16" t="s">
         <v>193</v>
       </c>
-      <c r="G24" s="15" t="s">
+      <c r="F24" s="16" t="s">
         <v>194</v>
       </c>
-      <c r="H24" s="15" t="s">
+      <c r="G24" s="16" t="s">
         <v>195</v>
       </c>
-      <c r="I24" s="15" t="s">
+      <c r="H24" s="16" t="s">
         <v>196</v>
+      </c>
+      <c r="I24" s="16" t="s">
+        <v>197</v>
       </c>
       <c r="J24" s="4">
         <v>5</v>
@@ -2408,139 +2465,139 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="16.282" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="18.71" bestFit="true" customWidth="true" style="0"/>
     <col min="2" max="2" width="15.139" bestFit="true" customWidth="true" style="0"/>
     <col min="3" max="3" width="12.854" bestFit="true" customWidth="true" style="0"/>
     <col min="4" max="4" width="42.275" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="31.707" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="50" customWidth="true" style="18"/>
+    <col min="5" max="5" width="32.992" bestFit="true" customWidth="true" style="0"/>
+    <col min="6" max="6" width="50" customWidth="true" style="19"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="19" t="s">
-        <v>197</v>
+      <c r="A1" s="20" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>2</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F3" s="14" t="s">
         <v>202</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>203</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="4" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>206</v>
-      </c>
-      <c r="F4" s="15" t="s">
         <v>207</v>
+      </c>
+      <c r="F4" s="16" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="5" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>8</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>211</v>
-      </c>
-      <c r="F5" s="16" t="s">
         <v>212</v>
+      </c>
+      <c r="F5" s="17" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="4" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>215</v>
-      </c>
-      <c r="F6" s="15" t="s">
-        <v>216</v>
+        <v>217</v>
+      </c>
+      <c r="F6" s="16" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C7" s="7" t="s">
         <v>8</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>219</v>
+        <v>70</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>220</v>
-      </c>
-      <c r="F7" s="16" t="s">
         <v>221</v>
+      </c>
+      <c r="F7" s="17" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="4" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>224</v>
+        <v>206</v>
       </c>
       <c r="E8" s="8" t="s">
         <v>225</v>
       </c>
-      <c r="F8" s="15" t="s">
+      <c r="F8" s="16" t="s">
         <v>226</v>
       </c>
     </row>
@@ -2555,32 +2612,32 @@
         <v>8</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>69</v>
+        <v>229</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>229</v>
-      </c>
-      <c r="F9" s="16" t="s">
         <v>230</v>
       </c>
+      <c r="F9" s="17" t="s">
+        <v>231</v>
+      </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="4" t="s">
-        <v>231</v>
+      <c r="A10" s="4">
+        <v>78941000.0</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>205</v>
+        <v>232</v>
       </c>
       <c r="E10" s="8" t="s">
         <v>233</v>
       </c>
-      <c r="F10" s="15" t="s">
+      <c r="F10" s="16" t="s">
         <v>234</v>
       </c>
     </row>
@@ -2589,384 +2646,384 @@
         <v>235</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>8</v>
       </c>
       <c r="D11" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>236</v>
+      </c>
+      <c r="F11" s="17" t="s">
         <v>237</v>
       </c>
-      <c r="E11" s="9" t="s">
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="4" t="s">
         <v>238</v>
       </c>
-      <c r="F11" s="16" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6">
-      <c r="A12" s="4">
-        <v>78941000.0</v>
-      </c>
       <c r="B12" s="6" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D12" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="F12" s="16" t="s">
         <v>240</v>
-      </c>
-      <c r="E12" s="8" t="s">
-        <v>241</v>
-      </c>
-      <c r="F12" s="15" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="5" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="C13" s="7" t="s">
         <v>8</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E13" s="9" t="s">
+        <v>243</v>
+      </c>
+      <c r="F13" s="17" t="s">
         <v>244</v>
-      </c>
-      <c r="F13" s="16" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="B14" s="6" t="s">
         <v>246</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>236</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>62</v>
+        <v>247</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>247</v>
-      </c>
-      <c r="F14" s="15" t="s">
         <v>248</v>
+      </c>
+      <c r="F14" s="16" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="5" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>8</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>46</v>
+        <v>252</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>251</v>
-      </c>
-      <c r="F15" s="16" t="s">
-        <v>252</v>
+        <v>253</v>
+      </c>
+      <c r="F15" s="17" t="s">
+        <v>254</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>236</v>
+        <v>251</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>254</v>
-      </c>
-      <c r="F16" s="15" t="s">
-        <v>255</v>
+        <v>256</v>
+      </c>
+      <c r="F16" s="16" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="5" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>236</v>
+        <v>259</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>92</v>
+        <v>260</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>257</v>
-      </c>
-      <c r="F17" s="16" t="s">
-        <v>258</v>
+        <v>261</v>
+      </c>
+      <c r="F17" s="17" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="4" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>250</v>
+        <v>264</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>92</v>
+        <v>124</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>260</v>
-      </c>
-      <c r="F18" s="15" t="s">
-        <v>261</v>
+        <v>265</v>
+      </c>
+      <c r="F18" s="16" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="5" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="C19" s="7" t="s">
         <v>14</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>84</v>
+        <v>269</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>264</v>
-      </c>
-      <c r="F19" s="16" t="s">
-        <v>265</v>
+        <v>270</v>
+      </c>
+      <c r="F19" s="17" t="s">
+        <v>271</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="4" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>14</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>269</v>
-      </c>
-      <c r="F20" s="15" t="s">
-        <v>270</v>
+        <v>275</v>
+      </c>
+      <c r="F20" s="16" t="s">
+        <v>276</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="5" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>267</v>
+        <v>278</v>
       </c>
       <c r="C21" s="7" t="s">
         <v>14</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>272</v>
+        <v>138</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>273</v>
-      </c>
-      <c r="F21" s="16" t="s">
-        <v>274</v>
+        <v>279</v>
+      </c>
+      <c r="F21" s="17" t="s">
+        <v>280</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="4" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="C22" s="6" t="s">
         <v>14</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>277</v>
+        <v>138</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>278</v>
-      </c>
-      <c r="F22" s="15" t="s">
-        <v>279</v>
+        <v>282</v>
+      </c>
+      <c r="F22" s="16" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="5" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>276</v>
+        <v>285</v>
       </c>
       <c r="C23" s="7" t="s">
         <v>14</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>69</v>
+        <v>138</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>281</v>
-      </c>
-      <c r="F23" s="16" t="s">
-        <v>282</v>
+        <v>286</v>
+      </c>
+      <c r="F23" s="17" t="s">
+        <v>287</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="4" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>276</v>
+        <v>289</v>
       </c>
       <c r="C24" s="6" t="s">
         <v>14</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>92</v>
+        <v>146</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>284</v>
-      </c>
-      <c r="F24" s="15" t="s">
-        <v>285</v>
+        <v>290</v>
+      </c>
+      <c r="F24" s="16" t="s">
+        <v>291</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="5" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="C25" s="7" t="s">
         <v>14</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>288</v>
+        <v>146</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>289</v>
-      </c>
-      <c r="F25" s="16" t="s">
-        <v>290</v>
+        <v>294</v>
+      </c>
+      <c r="F25" s="17" t="s">
+        <v>295</v>
       </c>
     </row>
     <row r="26" spans="1:6">
-      <c r="A26" s="4" t="s">
-        <v>291</v>
+      <c r="A26" s="4">
+        <v>2317584</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C26" s="6" t="s">
         <v>14</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>123</v>
+        <v>146</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>293</v>
-      </c>
-      <c r="F26" s="15" t="s">
-        <v>294</v>
+        <v>296</v>
+      </c>
+      <c r="F26" s="16" t="s">
+        <v>297</v>
       </c>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="5" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>297</v>
-      </c>
-      <c r="F27" s="16" t="s">
-        <v>298</v>
+        <v>300</v>
+      </c>
+      <c r="F27" s="17" t="s">
+        <v>301</v>
       </c>
     </row>
     <row r="28" spans="1:6">
       <c r="A28" s="4" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>300</v>
-      </c>
-      <c r="F28" s="15" t="s">
-        <v>301</v>
+        <v>304</v>
+      </c>
+      <c r="F28" s="16" t="s">
+        <v>305</v>
       </c>
     </row>
     <row r="29" spans="1:6">
       <c r="A29" s="5" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="C29" s="7" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>145</v>
+        <v>160</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>304</v>
-      </c>
-      <c r="F29" s="16" t="s">
-        <v>305</v>
+        <v>308</v>
+      </c>
+      <c r="F29" s="17" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="30" spans="1:6">
-      <c r="A30" s="4" t="s">
-        <v>306</v>
+      <c r="A30" s="4">
+        <v>4771200000000.0</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>307</v>
@@ -2975,193 +3032,253 @@
         <v>19</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>145</v>
+        <v>160</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>308</v>
-      </c>
-      <c r="F30" s="15" t="s">
-        <v>309</v>
+        <v>310</v>
+      </c>
+      <c r="F30" s="16" t="s">
+        <v>311</v>
       </c>
     </row>
     <row r="31" spans="1:6">
       <c r="A31" s="5">
-        <v>2317584</v>
+        <v>1805628</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="C31" s="7" t="s">
         <v>19</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>145</v>
+        <v>313</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>310</v>
-      </c>
-      <c r="F31" s="16" t="s">
-        <v>311</v>
+        <v>314</v>
+      </c>
+      <c r="F31" s="17" t="s">
+        <v>315</v>
       </c>
     </row>
     <row r="32" spans="1:6">
       <c r="A32" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="B32" s="6" t="s">
         <v>312</v>
-      </c>
-      <c r="B32" s="6" t="s">
-        <v>313</v>
       </c>
       <c r="C32" s="6" t="s">
         <v>19</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>145</v>
+        <v>160</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>314</v>
-      </c>
-      <c r="F32" s="15" t="s">
-        <v>315</v>
+        <v>317</v>
+      </c>
+      <c r="F32" s="16" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="33" spans="1:6">
       <c r="A33" s="5" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>317</v>
+        <v>312</v>
       </c>
       <c r="C33" s="7" t="s">
         <v>19</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>318</v>
-      </c>
-      <c r="F33" s="16" t="s">
-        <v>319</v>
+        <v>320</v>
+      </c>
+      <c r="F33" s="17" t="s">
+        <v>321</v>
       </c>
     </row>
     <row r="34" spans="1:6">
       <c r="A34" s="4" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>317</v>
+        <v>312</v>
       </c>
       <c r="C34" s="6" t="s">
         <v>19</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>321</v>
-      </c>
-      <c r="F34" s="15" t="s">
-        <v>322</v>
+        <v>323</v>
+      </c>
+      <c r="F34" s="16" t="s">
+        <v>324</v>
       </c>
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="5" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>324</v>
+        <v>312</v>
       </c>
       <c r="C35" s="7" t="s">
         <v>19</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>326</v>
-      </c>
-      <c r="F35" s="16" t="s">
         <v>327</v>
+      </c>
+      <c r="F35" s="17" t="s">
+        <v>328</v>
       </c>
     </row>
     <row r="36" spans="1:6">
       <c r="A36" s="4" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C36" s="6" t="s">
         <v>19</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>183</v>
+        <v>331</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>330</v>
-      </c>
-      <c r="F36" s="15" t="s">
-        <v>331</v>
+        <v>332</v>
+      </c>
+      <c r="F36" s="16" t="s">
+        <v>333</v>
       </c>
     </row>
     <row r="37" spans="1:6">
       <c r="A37" s="5" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C37" s="7" t="s">
         <v>19</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>183</v>
+        <v>335</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>333</v>
-      </c>
-      <c r="F37" s="16" t="s">
-        <v>334</v>
+        <v>336</v>
+      </c>
+      <c r="F37" s="17" t="s">
+        <v>337</v>
       </c>
     </row>
     <row r="38" spans="1:6">
       <c r="A38" s="4" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="C38" s="6" t="s">
         <v>19</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>183</v>
+        <v>340</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>337</v>
-      </c>
-      <c r="F38" s="15" t="s">
-        <v>338</v>
+        <v>341</v>
+      </c>
+      <c r="F38" s="16" t="s">
+        <v>342</v>
       </c>
     </row>
     <row r="39" spans="1:6">
       <c r="A39" s="5" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>336</v>
+        <v>344</v>
       </c>
       <c r="C39" s="7" t="s">
         <v>19</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>240</v>
+        <v>184</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>340</v>
-      </c>
-      <c r="F39" s="16" t="s">
-        <v>341</v>
+        <v>345</v>
+      </c>
+      <c r="F39" s="17" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6">
+      <c r="A40" s="4" t="s">
+        <v>347</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>344</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="E40" s="8" t="s">
+        <v>348</v>
+      </c>
+      <c r="F40" s="16" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6">
+      <c r="A41" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="B41" s="7" t="s">
+        <v>351</v>
+      </c>
+      <c r="C41" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="E41" s="9" t="s">
+        <v>352</v>
+      </c>
+      <c r="F41" s="17" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
+      <c r="A42" s="4" t="s">
+        <v>354</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>351</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="E42" s="8" t="s">
+        <v>355</v>
+      </c>
+      <c r="F42" s="16" t="s">
+        <v>356</v>
       </c>
     </row>
   </sheetData>

</xml_diff>